<commit_message>
feat: enrich data test
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/ORDER_TEST_DATA.xlsx
+++ b/src/test/resources/testdata/ORDER_TEST_DATA.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11472" windowHeight="9264"/>
+    <workbookView windowWidth="11472" windowHeight="9264" firstSheet="2" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCT_DETAIL_PAGE" sheetId="1" r:id="rId1"/>
@@ -73,13 +73,10 @@
     <t>M</t>
   </si>
   <si>
-    <t>https://theblues.com.vn/san-pham/ao-nam-the-thao-co-tron-tvm-t1s-22-711/</t>
-  </si>
-  <si>
-    <t>Áo Nam Thể Thao Cổ Trơn TVM-T1S/22-711</t>
-  </si>
-  <si>
-    <t>179000</t>
+    <t>https://theblues.com.vn/san-pham/quan-jeans-nam-dai-bjmgt2019-12-black/</t>
+  </si>
+  <si>
+    <t>Quần jeans Nam Dài BJMGT2019-12-BLACK</t>
   </si>
   <si>
     <t>TC_AC_2</t>
@@ -106,6 +103,9 @@
     <t>TC_AC_5</t>
   </si>
   <si>
+    <t>https://theblues.com.vn/san-pham/ao-can-ban-nu-hfa1211-t2s-23-779/</t>
+  </si>
+  <si>
     <t>METHOD</t>
   </si>
   <si>
@@ -211,7 +211,7 @@
     <t>0232324234</t>
   </si>
   <si>
-    <t>hellobitches@example.com</t>
+    <t>normng@example.com</t>
   </si>
   <si>
     <t>128 TT</t>
@@ -270,11 +270,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="0.00_);[Red]\(0.00\)"/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -323,15 +323,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="13"/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -346,23 +339,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -378,22 +355,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -415,10 +384,49 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -428,14 +436,6 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -446,97 +446,175 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -549,84 +627,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -649,11 +649,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -674,16 +680,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -705,15 +711,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -723,17 +720,20 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -742,82 +742,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -826,55 +826,55 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -903,7 +903,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="48">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
@@ -1323,10 +1323,10 @@
         <v>19</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="F4">
+        <v>29</v>
       </c>
       <c r="H4">
         <v>10</v>
@@ -1334,10 +1334,10 @@
     </row>
     <row r="5" customFormat="1" ht="30" customHeight="1" spans="1:8">
       <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
         <v>21</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>14</v>
@@ -1346,7 +1346,7 @@
         <v>17</v>
       </c>
       <c r="G5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H5">
         <v>3</v>
@@ -1354,10 +1354,10 @@
     </row>
     <row r="6" customFormat="1" ht="30" customHeight="1" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>14</v>
@@ -1366,7 +1366,7 @@
         <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -1374,10 +1374,10 @@
     </row>
     <row r="7" customFormat="1" ht="30" customHeight="1" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>14</v>
@@ -1386,27 +1386,30 @@
         <v>17</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="1" ht="30" customHeight="1" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
+      <c r="C8" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="F8" t="s">
         <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" t="s">
-        <v>27</v>
+        <v>22</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:1">
@@ -1455,7 +1458,8 @@
     <hyperlink ref="C6" r:id="rId2" display="https://theblues.com.vn/san-pham/thun-croptop-in-hinh-tvm-t2m-19-478/"/>
     <hyperlink ref="C7" r:id="rId2" display="https://theblues.com.vn/san-pham/thun-croptop-in-hinh-tvm-t2m-19-478/"/>
     <hyperlink ref="C3" r:id="rId2" display="https://theblues.com.vn/san-pham/thun-croptop-in-hinh-tvm-t2m-19-478/"/>
-    <hyperlink ref="C4" r:id="rId3" display="https://theblues.com.vn/san-pham/ao-nam-the-thao-co-tron-tvm-t1s-22-711/" tooltip="https://theblues.com.vn/san-pham/ao-nam-the-thao-co-tron-tvm-t1s-22-711/"/>
+    <hyperlink ref="C4" r:id="rId3" display="https://theblues.com.vn/san-pham/quan-jeans-nam-dai-bjmgt2019-12-black/" tooltip="https://theblues.com.vn/san-pham/quan-jeans-nam-dai-bjmgt2019-12-black/"/>
+    <hyperlink ref="C8" r:id="rId4" display="https://theblues.com.vn/san-pham/ao-can-ban-nu-hfa1211-t2s-23-779/"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1517,7 +1521,7 @@
         <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
         <v>36</v>
@@ -1735,7 +1739,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
         <v>62</v>
@@ -1765,14 +1769,14 @@
         <v>67</v>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1"/>
-    <row r="5" ht="48" customHeight="1"/>
+    <row r="4" ht="48" hidden="1" customHeight="1"/>
+    <row r="5" ht="48" hidden="1" customHeight="1"/>
     <row r="6" customFormat="1" ht="48" customHeight="1" spans="2:12">
       <c r="B6" s="2" t="s">
         <v>71</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>72</v>
@@ -1807,7 +1811,7 @@
         <v>73</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>62</v>
@@ -1839,7 +1843,7 @@
         <v>74</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
         <v>62</v>
@@ -1872,7 +1876,7 @@
         <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
         <v>62</v>
@@ -1905,7 +1909,7 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" t="s">
         <v>62</v>
@@ -1940,7 +1944,7 @@
         <v>78</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
         <v>62</v>
@@ -1952,13 +1956,13 @@
         <v>64</v>
       </c>
       <c r="G11" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11">
-        <v>13</v>
+        <v>44</v>
+      </c>
+      <c r="I11" t="s">
+        <v>79</v>
       </c>
       <c r="J11" t="s">
         <v>65</v>
@@ -1981,7 +1985,7 @@
         <v>80</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
         <v>62</v>
@@ -2013,7 +2017,7 @@
         <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
         <v>62</v>
@@ -2045,14 +2049,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="hellobitches@example.com" tooltip="mailto:hellobitches@example.com"/>
-    <hyperlink ref="F3" r:id="rId1" display="invalid_email.com"/>
-    <hyperlink ref="F6" r:id="rId1" display="hellobitches@example.com" tooltip="mailto:hellobitches@example.com"/>
-    <hyperlink ref="F7" r:id="rId1" display="hellobitches@example.com" tooltip="mailto:hellobitches@example.com"/>
-    <hyperlink ref="F10" r:id="rId1" display="invalid_email.com" tooltip="mailto:hellobitches@example.com"/>
-    <hyperlink ref="F11" r:id="rId1" display="hellobitches@example.com" tooltip="mailto:hellobitches@example.com"/>
-    <hyperlink ref="F12" r:id="rId1" display="hellobitches@example.com" tooltip="mailto:hellobitches@example.com"/>
-    <hyperlink ref="F13" r:id="rId1" display="hellobitches@example.com" tooltip="mailto:hellobitches@example.com"/>
+    <hyperlink ref="F2" r:id="rId1" display="normng@example.com" tooltip="mailto:normng@example.com"/>
+    <hyperlink ref="F3" r:id="rId2" display="invalid_email.com"/>
+    <hyperlink ref="F6" r:id="rId1" display="normng@example.com" tooltip="mailto:normng@example.com"/>
+    <hyperlink ref="F7" r:id="rId1" display="normng@example.com" tooltip="mailto:normng@example.com"/>
+    <hyperlink ref="F10" r:id="rId2" display="invalid_email.com" tooltip="mailto:hellobitches@example.com"/>
+    <hyperlink ref="F11" r:id="rId1" display="normng@example.com" tooltip="mailto:normng@example.com"/>
+    <hyperlink ref="F12" r:id="rId1" display="normng@example.com" tooltip="mailto:normng@example.com"/>
+    <hyperlink ref="F13" r:id="rId1" display="normng@example.com" tooltip="mailto:normng@example.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>